<commit_message>
Fail fast with 409 when leads file is locked by Excel
Probe write access (and check for Excel's ~$ lock file) before running
SerpAPI calls so we don't burn credits when the file is open.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tustin Group Lead Gen list.xlsx
+++ b/Tustin Group Lead Gen list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH1000"/>
+  <dimension ref="A1:AK1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="32" customWidth="1" style="11" min="1" max="1"/>
@@ -569,29 +569,44 @@
           <t>Industry</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="0" t="inlineStr">
         <is>
           <t>Enriched_Website</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="0" t="inlineStr">
         <is>
           <t>Enriched_LinkedIn</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="0" t="inlineStr">
         <is>
           <t>Enriched_Title</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="0" t="inlineStr">
         <is>
           <t>Enriched_Description</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="0" t="inlineStr">
         <is>
           <t>Enriched_Location</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>Enriched_LinkedIn_Headline</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>Enriched_LinkedIn_Summary</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>Enriched_LinkedIn_Company_Description</t>
         </is>
       </c>
     </row>
@@ -683,23 +698,26 @@
       <c r="AA2" s="4" t="n"/>
       <c r="AB2" s="4" t="n"/>
       <c r="AC2" s="4" t="n"/>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>https://www.westtown.edu/</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t>Westtown School is a Quaker, coeducational, college preparatory day and boarding school for students in pre-kindergarten through twelfth grade.</t>
-        </is>
-      </c>
-      <c r="AH2" t="inlineStr">
+      <c r="AD2" s="0" t="inlineStr">
+        <is>
+          <t>https://www.westtown.edu/teacher/leigh-guarino/</t>
+        </is>
+      </c>
+      <c r="AE2" s="0" t="inlineStr"/>
+      <c r="AF2" s="0" t="inlineStr"/>
+      <c r="AG2" s="0" t="inlineStr">
+        <is>
+          <t>Physical Education · Student Support · Social-Emotional Learning  975 Westtown Road West Chester, PA 19382</t>
+        </is>
+      </c>
+      <c r="AH2" s="0" t="inlineStr">
         <is>
           <t>West Chester, PA</t>
         </is>
       </c>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
+      <c r="AK2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -789,6 +807,26 @@
       <c r="AA3" s="4" t="n"/>
       <c r="AB3" s="4" t="n"/>
       <c r="AC3" s="4" t="n"/>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>https://www.unitedlutheranseminary.edu/staff/alberto-dejesus</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>adejesus@uls.edu 215-248-7374</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>Avenue Philadelphia, PA</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr"/>
+      <c r="AK3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -878,6 +916,42 @@
       <c r="AA4" s="4" t="n"/>
       <c r="AB4" s="4" t="n"/>
       <c r="AC4" s="4" t="n"/>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>https://www4.lead411.com/Adam_Cheyney_31503377.html</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/adam-cheyney-53529136</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>Facilities Maintenance Engineer</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>Adam Cheyneyis the Facilities Maintenance Engineer of</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>Philadelphia, PA</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>Facilities Maintenance Engineer at ...</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>Experienced Facilities Engineer with a demonstrated history of working in the information technology and services industry.</t>
+        </is>
+      </c>
+      <c r="AK4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -967,6 +1041,26 @@
       <c r="AA5" s="4" t="n"/>
       <c r="AB5" s="4" t="n"/>
       <c r="AC5" s="4" t="n"/>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>https://rocketreach.co/adam-lord-email_38101037</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>Adam Lord, based in Harleysville, PA, US, is currently a Director of Operations at Deacon Industrial Supply Company</t>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>Harleysville, PA</t>
+        </is>
+      </c>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr"/>
+      <c r="AK5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -1052,6 +1146,26 @@
       <c r="AA6" s="4" t="n"/>
       <c r="AB6" s="4" t="n"/>
       <c r="AC6" s="4" t="n"/>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>https://www.lowermerion.org/departments/public-works-department/public-works-divisions/facilities-maintenance-division</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr"/>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>610-649-1022 Mission Statement Maintain all Township buildings with special emphasis on the improvement of energy conservation methods.</t>
+        </is>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>Avenue Ardmore, PA</t>
+        </is>
+      </c>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="inlineStr"/>
+      <c r="AK6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1141,6 +1255,26 @@
       <c r="AA7" s="4" t="n"/>
       <c r="AB7" s="4" t="n"/>
       <c r="AC7" s="4" t="n"/>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>https://www.gmahs.org/</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr"/>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>Gwynedd Mercy Academy High School is an independent, Catholic, all-girls preparatory high school that fosters academic rigor, personal growth,</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>Lower Gwynedd, PA</t>
+        </is>
+      </c>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr"/>
+      <c r="AK7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -1230,6 +1364,34 @@
       <c r="AA8" s="4" t="n"/>
       <c r="AB8" s="4" t="n"/>
       <c r="AC8" s="4" t="n"/>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>https://www.adapt.io/contact/alan-mitchell/188054403</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/alan-mitchell-3b964a4</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr"/>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>Alan Mitchell is the Operations Manager at Spitz, with a rich history in the Manufacturing, dating back to 1947</t>
+        </is>
+      </c>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>Spitz, Inc.</t>
+        </is>
+      </c>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>Experience: Spitz, Inc. · Location: Greater Philadelphia · 98 connections on LinkedIn. View Alan Mitchell's profile on LinkedIn, a professional community of 1</t>
+        </is>
+      </c>
+      <c r="AK8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1327,6 +1489,14 @@
       <c r="AA9" s="4" t="n"/>
       <c r="AB9" s="4" t="n"/>
       <c r="AC9" s="4" t="n"/>
+      <c r="AD9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr"/>
+      <c r="AG9" t="inlineStr"/>
+      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr"/>
+      <c r="AJ9" t="inlineStr"/>
+      <c r="AK9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1416,6 +1586,26 @@
       <c r="AA10" s="4" t="n"/>
       <c r="AB10" s="4" t="n"/>
       <c r="AC10" s="4" t="n"/>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>https://www2.afpm.org/forms/DirectoryListingSearch/view?id=25F3F0000000F1</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr"/>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>Curtiss-Wright, EST Group 2701 Township Line Road Hatfield, PA 19440</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>Road Hatfield, PA</t>
+        </is>
+      </c>
+      <c r="AI10" t="inlineStr"/>
+      <c r="AJ10" t="inlineStr"/>
+      <c r="AK10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add Copilot bot endpoints and LLM-powered enrichment intelligence
- /copilot/lookup, /brief, /respond for Teams Copilot Studio integration
- intelligence layer wires OpenRouter (Claude Haiku 4.5) + Tustin's 6 cold-call scripts
- enrichment now writes 8 new columns: tenure, prior companies, title qualifier, signal tag, opener
- OpenAPI spec at context/copilot_openapi.json for Copilot Studio upload

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tustin Group Lead Gen list.xlsx
+++ b/Tustin Group Lead Gen list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK1000"/>
+  <dimension ref="A1:AS1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="32" customWidth="1" style="11" min="1" max="1"/>
@@ -594,19 +594,59 @@
           <t>Enriched_Location</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AI1" s="0" t="inlineStr">
         <is>
           <t>Enriched_LinkedIn_Headline</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AJ1" s="0" t="inlineStr">
         <is>
           <t>Enriched_LinkedIn_Summary</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AK1" s="0" t="inlineStr">
         <is>
           <t>Enriched_LinkedIn_Company_Description</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>Enriched_Tenure_Months</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>Enriched_Tenure_Label</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>Enriched_Prior_Company_1</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>Enriched_Prior_Company_2</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>Enriched_Title_Qualifier</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>Enriched_Signal_Tag</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>Enriched_Script_Used</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>Enriched_Personalized_Opener</t>
         </is>
       </c>
     </row>
@@ -715,9 +755,37 @@
           <t>West Chester, PA</t>
         </is>
       </c>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
+      <c r="AI2" s="0" t="inlineStr"/>
+      <c r="AJ2" s="0" t="inlineStr"/>
+      <c r="AK2" s="0" t="inlineStr"/>
+      <c r="AL2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>IN_HOUSE</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>Script 6: Reactive</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>Hi Leigh, this is Matt from The Tustin Group — we're a commercial building services company working with schools and institutions across the greater Philadelphia area. I'm calling because most facilities teams like yours are managing HVAC, water treatment, and fire safety across multiple vendors on a reactive basis, and I wanted to see if a consolidated service agreement might reduce your total cost of ownership.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -807,26 +875,26 @@
       <c r="AA3" s="4" t="n"/>
       <c r="AB3" s="4" t="n"/>
       <c r="AC3" s="4" t="n"/>
-      <c r="AD3" t="inlineStr">
+      <c r="AD3" s="0" t="inlineStr">
         <is>
           <t>https://www.unitedlutheranseminary.edu/staff/alberto-dejesus</t>
         </is>
       </c>
-      <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr">
+      <c r="AE3" s="0" t="inlineStr"/>
+      <c r="AF3" s="0" t="inlineStr"/>
+      <c r="AG3" s="0" t="inlineStr">
         <is>
           <t>adejesus@uls.edu 215-248-7374</t>
         </is>
       </c>
-      <c r="AH3" t="inlineStr">
+      <c r="AH3" s="0" t="inlineStr">
         <is>
           <t>Avenue Philadelphia, PA</t>
         </is>
       </c>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr"/>
+      <c r="AI3" s="0" t="inlineStr"/>
+      <c r="AJ3" s="0" t="inlineStr"/>
+      <c r="AK3" s="0" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -916,42 +984,42 @@
       <c r="AA4" s="4" t="n"/>
       <c r="AB4" s="4" t="n"/>
       <c r="AC4" s="4" t="n"/>
-      <c r="AD4" t="inlineStr">
+      <c r="AD4" s="0" t="inlineStr">
         <is>
           <t>https://www4.lead411.com/Adam_Cheyney_31503377.html</t>
         </is>
       </c>
-      <c r="AE4" t="inlineStr">
+      <c r="AE4" s="0" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/adam-cheyney-53529136</t>
         </is>
       </c>
-      <c r="AF4" t="inlineStr">
+      <c r="AF4" s="0" t="inlineStr">
         <is>
           <t>Facilities Maintenance Engineer</t>
         </is>
       </c>
-      <c r="AG4" t="inlineStr">
+      <c r="AG4" s="0" t="inlineStr">
         <is>
           <t>Adam Cheyneyis the Facilities Maintenance Engineer of</t>
         </is>
       </c>
-      <c r="AH4" t="inlineStr">
+      <c r="AH4" s="0" t="inlineStr">
         <is>
           <t>Philadelphia, PA</t>
         </is>
       </c>
-      <c r="AI4" t="inlineStr">
+      <c r="AI4" s="0" t="inlineStr">
         <is>
           <t>Facilities Maintenance Engineer at ...</t>
         </is>
       </c>
-      <c r="AJ4" t="inlineStr">
+      <c r="AJ4" s="0" t="inlineStr">
         <is>
           <t>Experienced Facilities Engineer with a demonstrated history of working in the information technology and services industry.</t>
         </is>
       </c>
-      <c r="AK4" t="inlineStr"/>
+      <c r="AK4" s="0" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1041,26 +1109,26 @@
       <c r="AA5" s="4" t="n"/>
       <c r="AB5" s="4" t="n"/>
       <c r="AC5" s="4" t="n"/>
-      <c r="AD5" t="inlineStr">
+      <c r="AD5" s="0" t="inlineStr">
         <is>
           <t>https://rocketreach.co/adam-lord-email_38101037</t>
         </is>
       </c>
-      <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr">
+      <c r="AE5" s="0" t="inlineStr"/>
+      <c r="AF5" s="0" t="inlineStr"/>
+      <c r="AG5" s="0" t="inlineStr">
         <is>
           <t>Adam Lord, based in Harleysville, PA, US, is currently a Director of Operations at Deacon Industrial Supply Company</t>
         </is>
       </c>
-      <c r="AH5" t="inlineStr">
+      <c r="AH5" s="0" t="inlineStr">
         <is>
           <t>Harleysville, PA</t>
         </is>
       </c>
-      <c r="AI5" t="inlineStr"/>
-      <c r="AJ5" t="inlineStr"/>
-      <c r="AK5" t="inlineStr"/>
+      <c r="AI5" s="0" t="inlineStr"/>
+      <c r="AJ5" s="0" t="inlineStr"/>
+      <c r="AK5" s="0" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -1146,26 +1214,26 @@
       <c r="AA6" s="4" t="n"/>
       <c r="AB6" s="4" t="n"/>
       <c r="AC6" s="4" t="n"/>
-      <c r="AD6" t="inlineStr">
+      <c r="AD6" s="0" t="inlineStr">
         <is>
           <t>https://www.lowermerion.org/departments/public-works-department/public-works-divisions/facilities-maintenance-division</t>
         </is>
       </c>
-      <c r="AE6" t="inlineStr"/>
-      <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="inlineStr">
+      <c r="AE6" s="0" t="inlineStr"/>
+      <c r="AF6" s="0" t="inlineStr"/>
+      <c r="AG6" s="0" t="inlineStr">
         <is>
           <t>610-649-1022 Mission Statement Maintain all Township buildings with special emphasis on the improvement of energy conservation methods.</t>
         </is>
       </c>
-      <c r="AH6" t="inlineStr">
+      <c r="AH6" s="0" t="inlineStr">
         <is>
           <t>Avenue Ardmore, PA</t>
         </is>
       </c>
-      <c r="AI6" t="inlineStr"/>
-      <c r="AJ6" t="inlineStr"/>
-      <c r="AK6" t="inlineStr"/>
+      <c r="AI6" s="0" t="inlineStr"/>
+      <c r="AJ6" s="0" t="inlineStr"/>
+      <c r="AK6" s="0" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1255,26 +1323,26 @@
       <c r="AA7" s="4" t="n"/>
       <c r="AB7" s="4" t="n"/>
       <c r="AC7" s="4" t="n"/>
-      <c r="AD7" t="inlineStr">
+      <c r="AD7" s="0" t="inlineStr">
         <is>
           <t>https://www.gmahs.org/</t>
         </is>
       </c>
-      <c r="AE7" t="inlineStr"/>
-      <c r="AF7" t="inlineStr"/>
-      <c r="AG7" t="inlineStr">
+      <c r="AE7" s="0" t="inlineStr"/>
+      <c r="AF7" s="0" t="inlineStr"/>
+      <c r="AG7" s="0" t="inlineStr">
         <is>
           <t>Gwynedd Mercy Academy High School is an independent, Catholic, all-girls preparatory high school that fosters academic rigor, personal growth,</t>
         </is>
       </c>
-      <c r="AH7" t="inlineStr">
+      <c r="AH7" s="0" t="inlineStr">
         <is>
           <t>Lower Gwynedd, PA</t>
         </is>
       </c>
-      <c r="AI7" t="inlineStr"/>
-      <c r="AJ7" t="inlineStr"/>
-      <c r="AK7" t="inlineStr"/>
+      <c r="AI7" s="0" t="inlineStr"/>
+      <c r="AJ7" s="0" t="inlineStr"/>
+      <c r="AK7" s="0" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -1364,34 +1432,34 @@
       <c r="AA8" s="4" t="n"/>
       <c r="AB8" s="4" t="n"/>
       <c r="AC8" s="4" t="n"/>
-      <c r="AD8" t="inlineStr">
+      <c r="AD8" s="0" t="inlineStr">
         <is>
           <t>https://www.adapt.io/contact/alan-mitchell/188054403</t>
         </is>
       </c>
-      <c r="AE8" t="inlineStr">
+      <c r="AE8" s="0" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/alan-mitchell-3b964a4</t>
         </is>
       </c>
-      <c r="AF8" t="inlineStr"/>
-      <c r="AG8" t="inlineStr">
+      <c r="AF8" s="0" t="inlineStr"/>
+      <c r="AG8" s="0" t="inlineStr">
         <is>
           <t>Alan Mitchell is the Operations Manager at Spitz, with a rich history in the Manufacturing, dating back to 1947</t>
         </is>
       </c>
-      <c r="AH8" t="inlineStr"/>
-      <c r="AI8" t="inlineStr">
+      <c r="AH8" s="0" t="inlineStr"/>
+      <c r="AI8" s="0" t="inlineStr">
         <is>
           <t>Spitz, Inc.</t>
         </is>
       </c>
-      <c r="AJ8" t="inlineStr">
+      <c r="AJ8" s="0" t="inlineStr">
         <is>
           <t>Experience: Spitz, Inc. · Location: Greater Philadelphia · 98 connections on LinkedIn. View Alan Mitchell's profile on LinkedIn, a professional community of 1</t>
         </is>
       </c>
-      <c r="AK8" t="inlineStr"/>
+      <c r="AK8" s="0" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1489,14 +1557,14 @@
       <c r="AA9" s="4" t="n"/>
       <c r="AB9" s="4" t="n"/>
       <c r="AC9" s="4" t="n"/>
-      <c r="AD9" t="inlineStr"/>
-      <c r="AE9" t="inlineStr"/>
-      <c r="AF9" t="inlineStr"/>
-      <c r="AG9" t="inlineStr"/>
-      <c r="AH9" t="inlineStr"/>
-      <c r="AI9" t="inlineStr"/>
-      <c r="AJ9" t="inlineStr"/>
-      <c r="AK9" t="inlineStr"/>
+      <c r="AD9" s="0" t="inlineStr"/>
+      <c r="AE9" s="0" t="inlineStr"/>
+      <c r="AF9" s="0" t="inlineStr"/>
+      <c r="AG9" s="0" t="inlineStr"/>
+      <c r="AH9" s="0" t="inlineStr"/>
+      <c r="AI9" s="0" t="inlineStr"/>
+      <c r="AJ9" s="0" t="inlineStr"/>
+      <c r="AK9" s="0" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1586,26 +1654,26 @@
       <c r="AA10" s="4" t="n"/>
       <c r="AB10" s="4" t="n"/>
       <c r="AC10" s="4" t="n"/>
-      <c r="AD10" t="inlineStr">
+      <c r="AD10" s="0" t="inlineStr">
         <is>
           <t>https://www2.afpm.org/forms/DirectoryListingSearch/view?id=25F3F0000000F1</t>
         </is>
       </c>
-      <c r="AE10" t="inlineStr"/>
-      <c r="AF10" t="inlineStr"/>
-      <c r="AG10" t="inlineStr">
+      <c r="AE10" s="0" t="inlineStr"/>
+      <c r="AF10" s="0" t="inlineStr"/>
+      <c r="AG10" s="0" t="inlineStr">
         <is>
           <t>Curtiss-Wright, EST Group 2701 Township Line Road Hatfield, PA 19440</t>
         </is>
       </c>
-      <c r="AH10" t="inlineStr">
+      <c r="AH10" s="0" t="inlineStr">
         <is>
           <t>Road Hatfield, PA</t>
         </is>
       </c>
-      <c r="AI10" t="inlineStr"/>
-      <c r="AJ10" t="inlineStr"/>
-      <c r="AK10" t="inlineStr"/>
+      <c r="AI10" s="0" t="inlineStr"/>
+      <c r="AJ10" s="0" t="inlineStr"/>
+      <c r="AK10" s="0" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">

</xml_diff>